<commit_message>
Add collection labels and tests
</commit_message>
<xml_diff>
--- a/tadkaPending.xlsx
+++ b/tadkaPending.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -39,18 +39,6 @@
     <t xml:space="preserve">Basis for estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">OSC-8 hyperlinks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40–60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80–120 + 2–3 golden fixtures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small addition to Terminal.hs capability detection (like existing capNoColor/capForceColor) + conditional wrap in Graphical.hs. Test ratio follows TermColor.hs (2.3× code).</t>
-  </si>
-  <si>
     <t xml:space="preserve">Same-line multi-label packing</t>
   </si>
   <si>
@@ -106,15 +94,6 @@
   </si>
   <si>
     <t xml:space="preserve">Needs a new module wrapping an external Haskell highlighter, merging its output with existing label-color ANSI styling without clobbering carets. Heaviest dependency-integration item, as your own docs flag.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~790–1300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~660–1000</t>
   </si>
 </sst>
 </file>
@@ -129,6 +108,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -150,11 +130,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -204,19 +186,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -343,7 +325,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C7:G14"/>
+  <dimension ref="C7:G13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -363,7 +345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="2" t="n">
         <v>1</v>
       </c>
@@ -380,7 +362,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2" t="n">
         <v>2</v>
       </c>
@@ -397,7 +379,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="2" t="n">
         <v>3</v>
       </c>
@@ -408,30 +390,30 @@
         <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="2" t="n">
         <v>5</v>
       </c>
@@ -448,35 +430,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="3"/>
-      <c r="D14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" s="3"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
collection labels patch and tests
</commit_message>
<xml_diff>
--- a/tadkaPending.xlsx
+++ b/tadkaPending.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -39,18 +39,6 @@
     <t xml:space="preserve">Basis for estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">OSC-8 hyperlinks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40–60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80–120 + 2–3 golden fixtures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small addition to Terminal.hs capability detection (like existing capNoColor/capForceColor) + conditional wrap in Graphical.hs. Test ratio follows TermColor.hs (2.3× code).</t>
-  </si>
-  <si>
     <t xml:space="preserve">Same-line multi-label packing</t>
   </si>
   <si>
@@ -106,15 +94,6 @@
   </si>
   <si>
     <t xml:space="preserve">Needs a new module wrapping an external Haskell highlighter, merging its output with existing label-color ANSI styling without clobbering carets. Heaviest dependency-integration item, as your own docs flag.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~790–1300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~660–1000</t>
   </si>
 </sst>
 </file>
@@ -129,6 +108,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -150,11 +130,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -204,19 +186,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -343,7 +325,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C7:G14"/>
+  <dimension ref="C7:G13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -363,7 +345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="2" t="n">
         <v>1</v>
       </c>
@@ -380,7 +362,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2" t="n">
         <v>2</v>
       </c>
@@ -397,7 +379,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="2" t="n">
         <v>3</v>
       </c>
@@ -408,30 +390,30 @@
         <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="2" t="n">
         <v>5</v>
       </c>
@@ -448,35 +430,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="3"/>
-      <c r="D14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" s="3"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
build succeeded and tested with ghc 9.6.7
</commit_message>
<xml_diff>
--- a/tadkaPending.xlsx
+++ b/tadkaPending.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -49,18 +49,6 @@
   </si>
   <si>
     <t xml:space="preserve">This is a new lane-assignment engine on the horizontal axis, not an extension of Layout.hs — your own PENDING_WORK.md says so. Sized similarly to Layout.hs+LinePlan.hs combined (160 LOC) since it's comparable proof complexity, plus wiring into Graphical.hs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection labels in derive macro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60–100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60–100 + 2–4 compile-fail fixtures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context.hs already supports variable-length label lists — this is TH-layer only (new DiagnosticSpec field option, reify validation, dispatch through existing buildContextWith). Smaller than the base derive macro since it reuses existing plumbing.</t>
   </si>
   <si>
     <t xml:space="preserve">Lazy/file-backed SourceCode</t>
@@ -325,7 +313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C7:G13"/>
+  <dimension ref="C7:G12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -362,9 +350,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>9</v>
@@ -373,32 +361,32 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>16</v>
@@ -413,29 +401,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="3"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Verify build across GHC 9.6-9.14, drop 9.4.7 support
</commit_message>
<xml_diff>
--- a/tadkaPending.xlsx
+++ b/tadkaPending.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -49,18 +49,6 @@
   </si>
   <si>
     <t xml:space="preserve">This is a new lane-assignment engine on the horizontal axis, not an extension of Layout.hs — your own PENDING_WORK.md says so. Sized similarly to Layout.hs+LinePlan.hs combined (160 LOC) since it's comparable proof complexity, plus wiring into Graphical.hs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection labels in derive macro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60–100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60–100 + 2–4 compile-fail fixtures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context.hs already supports variable-length label lists — this is TH-layer only (new DiagnosticSpec field option, reify validation, dispatch through existing buildContextWith). Smaller than the base derive macro since it reuses existing plumbing.</t>
   </si>
   <si>
     <t xml:space="preserve">Lazy/file-backed SourceCode</t>
@@ -325,7 +313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C7:G13"/>
+  <dimension ref="C7:G12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -362,9 +350,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>9</v>
@@ -373,32 +361,32 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>16</v>
@@ -413,29 +401,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="3"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>